<commit_message>
chore(filiais): so as 3 limpas vao pro modelo da AIVA; INAPTA/nao consta ficam seguradas
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Filiais-modelo-AIVA-2026-09-18.xlsx
+++ b/docs/Filiais-modelo-AIVA-2026-09-18.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modelo AIVA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conferir antes de enviar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segurados (não enviar)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conferir antes de enviar" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Modelo AIVA'!$A$1:$O$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Modelo AIVA'!$A$1:$O$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -69,12 +70,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -447,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -548,72 +550,72 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Rei do Celular</t>
+          <t>Loja Contel - Santa Maria</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>35650000</t>
+          <t>97110800</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>DO PILAR</t>
+          <t>PREFEITO EVANDRO BEHR</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>3154</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>LOJA 105 107</t>
+          <t>SALA 09 COMERCIAL</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>CENTRO</t>
+          <t>CAMOBI</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>PITANGUI</t>
+          <t>SANTA MARIA</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>50072411000322</t>
+          <t>13337781000903</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>50072411000160</t>
+          <t>13337781000741</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Luiz Fernando Junio Lopes</t>
+          <t>Tiago Fagundes Brum</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>07883812610</t>
+          <t>00096974036</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>fvstylocell@gmail.com</t>
+          <t>curriculotiagofagundes@gmail.com</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>5567982228252</t>
+          <t>5555981071699</t>
         </is>
       </c>
     </row>
@@ -621,33 +623,33 @@
       <c r="A3" s="2" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>LF CELULARES LTDA.</t>
+          <t>FONEEXPRESS PARACATU</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>32340000</t>
+          <t>38600422</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>JOAO CESAR DE OLIVEIRA</t>
+          <t>JOAQUIM MURTINHO</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2792</t>
+          <t>21</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>ELDORADO</t>
+          <t>AMOREIRAS</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>CONTAGEM</t>
+          <t>PARACATU</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -657,32 +659,32 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>50072411000241</t>
+          <t>68182669000185</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>50072411000160</t>
+          <t>65870629000138</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Luiz Fernando Junio Lopes</t>
+          <t>Conrado Alves Pacheco</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>07883812610</t>
+          <t>11832778657</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>luizcellcg@gmail.com</t>
+          <t>drconradoalves@gmail.com</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>5564981835034</t>
+          <t>5538999132729</t>
         </is>
       </c>
     </row>
@@ -690,273 +692,402 @@
       <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Stylo Cell Itapema</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>FONEEXPRESS PARACATU</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>38600422</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>JOAQUIM MURTINHO</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>AMOREIRAS</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Itapema</t>
+          <t>PARACATU</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>46618959000277</t>
+          <t>68182669000185</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>46618959000196</t>
+          <t>65870629000138</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Felipe Aparecido da Silva Vianna</t>
+          <t>Lucas Alves Pacheco</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>05784977199</t>
+          <t>10138513660</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>felipeviannapro@gmail.com</t>
+          <t>lucaspaxeco@gmail.com</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>5567993518506</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Loja Contel - Santa Maria</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>97110800</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>PREFEITO EVANDRO BEHR</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>3154</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>SALA 09 COMERCIAL</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>CAMOBI</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>SANTA MARIA</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>RS</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>13337781000903</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>13337781000741</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Tiago Fagundes Brum</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>00096974036</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>curriculotiagofagundes@gmail.com</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>5555981071699</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>FONEEXPRESS PARACATU</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>38600422</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>JOAQUIM MURTINHO</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>AMOREIRAS</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>PARACATU</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>MG</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>68182669000185</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>65870629000138</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Conrado Alves Pacheco</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>11832778657</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>drconradoalves@gmail.com</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>5538999132729</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>FONEEXPRESS PARACATU</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>38600422</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>JOAQUIM MURTINHO</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>AMOREIRAS</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>PARACATU</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>MG</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>68182669000185</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>65870629000138</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Lucas Alves Pacheco</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>10138513660</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>lucaspaxeco@gmail.com</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
           <t>5538991292251</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O7"/>
+  <autoFilter ref="A1:O4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="80" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID VAREJO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>NOME DA LOJA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CEP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>LOGRADOURO</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>NÚMERO</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>COMPLEMENTO</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>BAIRRO</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>CIDADE</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>UF</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>CNPJ DA FILIAL</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>CNPJ DA MATRIZ</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>NOME COMPLETO</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>CPF (SÓ NUMEROS)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>TELEFONE (FORMATADO 55DDDTELEFONE)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>MOTIVO</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Rei do Celular</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>35650000</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>DO PILAR</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>119</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>LOJA 105 107</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>PITANGUI</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>50072411000322</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>50072411000160</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>Luiz Fernando Junio Lopes</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>07883812610</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>fvstylocell@gmail.com</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>5567982228252</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>situação na Receita: INAPTA · sem ID VAREJO na API da AIVA (loja ainda não existe lá) · controle interno: e-mail e DDD parecem ser da Stylo Cell; 9o digito incluido no telefone</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>LF CELULARES LTDA.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>32340000</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>JOAO CESAR DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>2792</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>ELDORADO</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>CONTAGEM</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>50072411000241</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>50072411000160</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Luiz Fernando Junio Lopes</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>07883812610</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>luizcellcg@gmail.com</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>5564981835034</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>situação na Receita: INAPTA · sem ID VAREJO na API da AIVA (loja ainda não existe lá) · controle interno: falta o nome da loja; 9o digito incluido no telefone; mesmo CPF da loja de Pitangui</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Stylo Cell Itapema</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Itapema</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>46618959000277</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>46618959000196</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Felipe Aparecido da Silva Vianna</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>05784977199</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>felipeviannapro@gmail.com</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>5567993518506</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Receita não respondeu / CNPJ não encontrado — endereço em branco · sem ID VAREJO na API da AIVA (loja ainda não existe lá)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -972,154 +1103,154 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Loja</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>CNPJ DA FILIAL</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Operador</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Avisos</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Rei do Celular</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>50072411000322</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Luiz Fernando Junio Lopes</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>situação na Receita: INAPTA · sem ID VAREJO na API da AIVA (loja ainda não existe lá) · controle interno: e-mail e DDD parecem ser da Stylo Cell; 9o digito incluido no telefone</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>LF CELULARES LTDA.</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>50072411000241</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Luiz Fernando Junio Lopes</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>situação na Receita: INAPTA · sem ID VAREJO na API da AIVA (loja ainda não existe lá) · controle interno: falta o nome da loja; 9o digito incluido no telefone; mesmo CPF da loja de Pitangui</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Stylo Cell Itapema</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>46618959000277</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Felipe Aparecido da Silva Vianna</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Receita não respondeu / CNPJ não encontrado — endereço em branco · sem ID VAREJO na API da AIVA (loja ainda não existe lá)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Loja Contel - Santa Maria</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>13337781000903</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Tiago Fagundes Brum</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>sem ID VAREJO na API da AIVA (loja ainda não existe lá) · matriz no portal: CONTEL TELECOM LTDA · controle interno: falta endereco completo (CEP, logradouro, numero, bairro)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>FONEEXPRESS PARACATU</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>68182669000185</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Conrado Alves Pacheco</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>sem ID VAREJO na API da AIVA (loja ainda não existe lá) · controle interno: matriz = FONEEXPRESS CRISTALINA; CEP 38600-422 e do bairro Amoreiras I, nao Centro</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>FONEEXPRESS PARACATU</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>68182669000185</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Lucas Alves Pacheco</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>sem ID VAREJO na API da AIVA (loja ainda não existe lá) · controle interno: 2o operador da mesma loja</t>
         </is>

</xml_diff>